<commit_message>
New updated codes, README not finished
</commit_message>
<xml_diff>
--- a/Experimental_data.xlsx
+++ b/Experimental_data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="PE_Normal"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="19">
   <si>
     <t>Time (hours)</t>
   </si>
@@ -58,6 +58,9 @@
     <t>Ammonia-deficient (repetition)</t>
   </si>
   <si>
+    <t>N (original)</t>
+  </si>
+  <si>
     <t>Time (Hours)</t>
   </si>
   <si>
@@ -83,7 +86,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="165" formatCode="#,##0.000000000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00000000"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -153,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="32">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -185,7 +192,25 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -212,8 +237,23 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -517,563 +557,579 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="16" width="12.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="17" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="17" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="17" width="14.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="17" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="18" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="18" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="19" width="12.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="24" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="30" width="13.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="30" width="16.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="30" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="30" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="30" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="30" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="30" width="15.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="30" width="15.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="30" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="30" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="30" width="15.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="30" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="31" width="13.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="31" width="13.290714285714287" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="F1" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" s="2" t="s">
+      <c r="I1" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="L1" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="13"/>
+      <c r="O1" s="26" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="4">
         <v>0</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="27">
         <v>0.228519</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="27">
         <v>274981.8993164774</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="27">
         <v>0.0011010000000000002</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="27">
         <v>5.389066666666667</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="27">
         <v>26.989574736966443</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="27">
         <v>0.1111325684836706</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="27">
         <v>0.9507718666666666</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="27">
         <v>866.3250567232511</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="27">
         <v>0.01961547976576436</v>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="27">
         <v>7.156666666666666</v>
       </c>
-      <c r="L2" s="5">
+      <c r="L2" s="27">
         <v>30000.00000000128</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2" s="27">
         <v>0.0033333333333332624</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="27">
         <f>10^-K2</f>
       </c>
-      <c r="O2" s="5">
+      <c r="O2" s="27">
         <v>0.00776378486929085</v>
       </c>
-      <c r="P2" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="5">
         <v>3.5</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="27">
         <v>0.234024</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="27">
         <v>1</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="27">
         <v>0</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="27">
         <v>5.336833333333334</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="27">
         <v>61.815993157381655</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="27">
         <v>0.07343260704739946</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="27">
         <v>0.9060905666666667</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="27">
         <v>281.8480451553724</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="27">
         <v>0.03438997492396747</v>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="27">
         <v>7.133333333333333</v>
       </c>
-      <c r="L3" s="5">
+      <c r="L3" s="27">
         <v>7500.00000000032</v>
       </c>
-      <c r="M3" s="5">
+      <c r="M3" s="27">
         <v>0.006666666666666525</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="27">
         <f>10^-K3</f>
       </c>
-      <c r="O3" s="5">
+      <c r="O3" s="27">
         <v>0.100931477902668</v>
       </c>
-      <c r="P3" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="4">
         <v>7</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="27">
         <v>0.27476100000000003</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="27">
         <v>274981.8993164774</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="27">
         <v>0.0011010000000000002</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="27">
         <v>5.513633333333334</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="27">
         <v>392.6398354053797</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="27">
         <v>0.029136822826870593</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="27">
         <v>0.9503526</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="27">
         <v>180.00148783408602</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="27">
         <v>0.04303297044178258</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="27">
         <v>7.066666666666666</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="27">
         <v>29999.999999995947</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="27">
         <v>0.0033333333333335586</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="27">
         <f>10^-K4</f>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="27">
         <v>0.293478233055139</v>
       </c>
-      <c r="P4" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="4">
         <v>16</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="27">
         <v>0.565425</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="27">
         <v>2749.8189931647744</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="27">
         <v>0.011010000000000002</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="27">
         <v>4.751833333333334</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="27">
         <v>64.51107913273023</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="27">
         <v>0.07188234213707226</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="27">
         <v>0.9042199333333333</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="27">
         <v>1329.3132097492294</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="27">
         <v>0.015835278738977443</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="27">
         <v>6.696666666666666</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="27">
         <v>1578.947368421061</v>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="27">
         <v>0.01452966314513554</v>
       </c>
-      <c r="N5" s="5">
+      <c r="N5" s="27">
         <f>10^-K5</f>
       </c>
-      <c r="O5" s="5">
+      <c r="O5" s="27">
         <v>1.67236008994913</v>
       </c>
-      <c r="P5" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="5">
         <v>19.5</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="27">
         <v>0.8351699999999999</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="27">
         <v>3666.4253242197233</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="27">
         <v>0.00953493969566664</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="27">
         <v>4.433533333333333</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="27">
         <v>23.962976243185217</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="27">
         <v>0.11794213741397849</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="27">
         <v>0.9334535333333333</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="27">
         <v>552.7568485761628</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="27">
         <v>0.02455683016028559</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="27">
         <v>6.513333333333333</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="27">
         <v>7500.00000000032</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="27">
         <v>0.006666666666666525</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6" s="27">
         <f>10^-K6</f>
       </c>
-      <c r="O6" s="5">
+      <c r="O6" s="27">
         <v>2.6288819279753</v>
       </c>
-      <c r="P6" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="4">
         <v>23</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="27">
         <v>1.02234</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="27">
         <v>180.31599955178834</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="27">
         <v>0.042995424465866156</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="27">
         <v>3.930066666666667</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="27">
         <v>10.698745404487646</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="27">
         <v>0.1765114758623674</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="27">
         <v>0.9368756666666666</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="27">
         <v>631.0361611826196</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="27">
         <v>0.022983292762231513</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="27">
         <v>6.363333333333333</v>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="27">
         <v>2307.692307692296</v>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="27">
         <v>0.012018504251546663</v>
       </c>
-      <c r="N7" s="5">
+      <c r="N7" s="27">
         <f>10^-K7</f>
       </c>
-      <c r="O7" s="5">
+      <c r="O7" s="27">
         <v>3.3059004025761</v>
       </c>
-      <c r="P7" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="4">
         <v>24</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="27">
         <v>1.06638</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="27">
         <v>916.6063310549247</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="27">
         <v>0.019069879391333342</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="27">
         <v>3.8788</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="27">
         <v>24.114183552824695</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="27">
         <v>0.11757177949377694</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="27">
         <v>0.9113481333333334</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="27">
         <v>11232.366445934198</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="27">
         <v>0.005447581557086704</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="27">
         <v>6.41</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="27">
         <v>10000.000000000426</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="27">
         <v>0.005773502691896135</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="27">
         <f>10^-K8</f>
       </c>
-      <c r="O8" s="5">
+      <c r="O8" s="27">
         <v>3.31832285642229</v>
       </c>
-      <c r="P8" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="5">
         <v>27.5</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="27">
         <v>1.2370349999999999</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="27">
         <v>255.7971156432352</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="27">
         <v>0.03609869907628249</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="27">
         <v>3.5394</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="27">
         <v>51.87881730822608</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="27">
         <v>0.08015753239714904</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="27">
         <v>0.9227773666666667</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="27">
         <v>667.9835477964043</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="27">
         <v>0.022338627671691095</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="27">
         <v>6.349999999999999</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="27">
         <v>9999.999999999538</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="27">
         <v>0.0057735026918963915</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="27">
         <f>10^-K9</f>
       </c>
-      <c r="O9" s="5">
+      <c r="O9" s="27">
         <v>3.33074516810587</v>
       </c>
-      <c r="P9" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="4">
         <v>31</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="27">
         <v>1.446225</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="27">
         <v>523.7750463170993</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="27">
         <v>0.025227079200731917</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="27">
         <v>3.2052333333333336</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="27">
         <v>56.593597415408176</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="27">
         <v>0.07674599519048388</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="27">
         <v>0.8364228666666667</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="27">
         <v>314.404712933345</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="27">
         <v>0.03256078366902601</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="27">
         <v>6.29</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="27">
         <v>10000.000000000426</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="27">
         <v>0.005773502691896135</v>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="27">
         <f>10^-K10</f>
       </c>
-      <c r="O10" s="5">
+      <c r="O10" s="27">
         <v>3.34937870671255</v>
       </c>
-      <c r="P10" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="4"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-      <c r="P11" s="6"/>
+      <c r="A11" s="5">
+        <v>40</v>
+      </c>
+      <c r="B11" s="27">
+        <v>1.1874900000000002</v>
+      </c>
+      <c r="C11" s="27">
+        <v>392.8312847378241</v>
+      </c>
+      <c r="D11" s="27">
+        <v>0.029129721934821176</v>
+      </c>
+      <c r="E11" s="27">
+        <v>3.885866666666667</v>
+      </c>
+      <c r="F11" s="27">
+        <v>6.722364895702947</v>
+      </c>
+      <c r="G11" s="27">
+        <v>0.2226785226384541</v>
+      </c>
+      <c r="H11" s="27">
+        <v>0.90749</v>
+      </c>
+      <c r="I11" s="27">
+        <v>631.4888749500838</v>
+      </c>
+      <c r="J11" s="27">
+        <v>0.022975052934940832</v>
+      </c>
+      <c r="K11" s="27">
+        <v>6.326666666666667</v>
+      </c>
+      <c r="L11" s="27">
+        <v>1874.9999999999966</v>
+      </c>
+      <c r="M11" s="27">
+        <v>0.013333333333333346</v>
+      </c>
+      <c r="N11" s="27">
+        <f>10^-K11</f>
+      </c>
+      <c r="O11" s="27">
+        <v>3.36801224531922</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="14"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
-      <c r="M12" s="20"/>
-      <c r="N12" s="15"/>
-      <c r="O12" s="15"/>
-      <c r="P12" s="13"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="28"/>
+      <c r="L12" s="28"/>
+      <c r="M12" s="28"/>
+      <c r="N12" s="29"/>
+      <c r="O12" s="29"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="14"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
-      <c r="M13" s="20"/>
-      <c r="N13" s="15"/>
-      <c r="O13" s="15"/>
-      <c r="P13" s="13"/>
+      <c r="A13" s="21"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="28"/>
+      <c r="L13" s="28"/>
+      <c r="M13" s="28"/>
+      <c r="N13" s="29"/>
+      <c r="O13" s="29"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="14"/>
+      <c r="A14" s="21"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -1086,9 +1142,8 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
-      <c r="N14" s="15"/>
-      <c r="O14" s="15"/>
-      <c r="P14" s="13"/>
+      <c r="N14" s="29"/>
+      <c r="O14" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1494,32 +1549,32 @@
   <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="16" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="18" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="18" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="19" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="22" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="24" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="24" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="25" width="14.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="12" t="s">
-        <v>11</v>
+      <c r="A1" s="18" t="s">
+        <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -1528,7 +1583,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
@@ -1537,7 +1592,7 @@
         <v>4</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>2</v>
@@ -1546,7 +1601,7 @@
         <v>5</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>2</v>
@@ -1555,7 +1610,7 @@
         <v>6</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -1601,7 +1656,7 @@
       <c r="N2" s="5">
         <f>10^-K2</f>
       </c>
-      <c r="O2" s="13"/>
+      <c r="O2" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="5">
@@ -1646,7 +1701,7 @@
       <c r="N3" s="5">
         <f>10^-K3</f>
       </c>
-      <c r="O3" s="13"/>
+      <c r="O3" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="4">
@@ -1691,7 +1746,7 @@
       <c r="N4" s="5">
         <f>10^-K4</f>
       </c>
-      <c r="O4" s="13"/>
+      <c r="O4" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="4">
@@ -1736,7 +1791,7 @@
       <c r="N5" s="5">
         <f>10^-K5</f>
       </c>
-      <c r="O5" s="13"/>
+      <c r="O5" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="5">
@@ -1781,7 +1836,7 @@
       <c r="N6" s="5">
         <f>10^-K6</f>
       </c>
-      <c r="O6" s="13"/>
+      <c r="O6" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="4">
@@ -1826,7 +1881,7 @@
       <c r="N7" s="5">
         <f>10^-K7</f>
       </c>
-      <c r="O7" s="13"/>
+      <c r="O7" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="4">
@@ -1871,7 +1926,7 @@
       <c r="N8" s="5">
         <f>10^-K8</f>
       </c>
-      <c r="O8" s="13"/>
+      <c r="O8" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="5">
@@ -1916,7 +1971,7 @@
       <c r="N9" s="5">
         <f>10^-K9</f>
       </c>
-      <c r="O9" s="13"/>
+      <c r="O9" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="4">
@@ -1961,7 +2016,7 @@
       <c r="N10" s="5">
         <f>10^-K10</f>
       </c>
-      <c r="O10" s="13"/>
+      <c r="O10" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="4">
@@ -2007,11 +2062,11 @@
         <f>10^-K11</f>
       </c>
       <c r="O11" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="14"/>
+      <c r="A12" s="20"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -2023,9 +2078,9 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="15"/>
-      <c r="N12" s="15"/>
-      <c r="O12" s="13"/>
+      <c r="M12" s="21"/>
+      <c r="N12" s="21"/>
+      <c r="O12" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2058,14 +2113,14 @@
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="12" t="s">
-        <v>11</v>
+      <c r="A1" s="18" t="s">
+        <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -2074,7 +2129,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
@@ -2083,7 +2138,7 @@
         <v>4</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>2</v>
@@ -2092,7 +2147,7 @@
         <v>5</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>2</v>
@@ -2101,7 +2156,7 @@
         <v>6</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -2553,7 +2608,7 @@
         <f>10^-K11</f>
       </c>
       <c r="O11" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2587,14 +2642,14 @@
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="12" t="s">
-        <v>11</v>
+      <c r="A1" s="18" t="s">
+        <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -2603,7 +2658,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
@@ -2612,7 +2667,7 @@
         <v>4</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>2</v>
@@ -2621,7 +2676,7 @@
         <v>5</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>2</v>
@@ -2630,7 +2685,7 @@
         <v>6</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -3082,7 +3137,7 @@
         <f>10^-K11</f>
       </c>
       <c r="O11" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -3116,14 +3171,14 @@
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="12" t="s">
-        <v>11</v>
+      <c r="A1" s="18" t="s">
+        <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -3132,7 +3187,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
@@ -3141,7 +3196,7 @@
         <v>4</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>2</v>
@@ -3150,7 +3205,7 @@
         <v>5</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>2</v>
@@ -3159,7 +3214,7 @@
         <v>6</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -3611,7 +3666,7 @@
         <f>10^-K11</f>
       </c>
       <c r="O11" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3624,24 +3679,25 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="16" width="14.147857142857141" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3656,7 +3712,7 @@
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -3668,10 +3724,13 @@
       <c r="I1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="12" t="s">
         <v>6</v>
       </c>
       <c r="K1" s="3"/>
+      <c r="L1" s="11" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="4">
@@ -3689,7 +3748,7 @@
       <c r="E2" s="5">
         <v>0.067418131422077</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="13">
         <v>1.0266189000000001</v>
       </c>
       <c r="G2" s="5">
@@ -3701,10 +3760,13 @@
       <c r="I2" s="5">
         <v>0.006666666666666821</v>
       </c>
-      <c r="J2" s="5">
-        <f>10^-G2</f>
+      <c r="J2" s="14">
+        <f>10^-H2</f>
       </c>
       <c r="K2" s="3"/>
+      <c r="L2" s="13">
+        <v>1.0266189000000001</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="4">
@@ -3722,7 +3784,7 @@
       <c r="E3" s="5">
         <v>0.044008572397255016</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="13">
         <v>0.9814482666666665</v>
       </c>
       <c r="G3" s="5">
@@ -3734,10 +3796,13 @@
       <c r="I3" s="5">
         <v>0.0033333333333332624</v>
       </c>
-      <c r="J3" s="5">
-        <f>10^-G3</f>
+      <c r="J3" s="14">
+        <f>10^-H3</f>
       </c>
       <c r="K3" s="3"/>
+      <c r="L3" s="13">
+        <v>0.9814482666666665</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="4">
@@ -3755,7 +3820,7 @@
       <c r="E4" s="5">
         <v>0.030120996737233625</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="13">
         <v>0.9563208</v>
       </c>
       <c r="G4" s="5">
@@ -3767,10 +3832,13 @@
       <c r="I4" s="5">
         <v>6.2803698347351e-16</v>
       </c>
-      <c r="J4" s="5">
-        <f>10^-G4</f>
+      <c r="J4" s="14">
+        <f>10^-H4</f>
       </c>
       <c r="K4" s="3"/>
+      <c r="L4" s="13">
+        <v>0.9563208</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="5">
@@ -3788,7 +3856,7 @@
       <c r="E5" s="5">
         <v>0.02594635491419437</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="13">
         <v>0.9399317666666667</v>
       </c>
       <c r="G5" s="5">
@@ -3800,10 +3868,13 @@
       <c r="I5" s="5">
         <v>6.2803698347351e-16</v>
       </c>
-      <c r="J5" s="5">
-        <f>10^-G5</f>
+      <c r="J5" s="14">
+        <f>10^-H5</f>
       </c>
       <c r="K5" s="3"/>
+      <c r="L5" s="13">
+        <v>0.9399317666666667</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="4">
@@ -3821,8 +3892,8 @@
       <c r="E6" s="5">
         <v>0.0675168456345856</v>
       </c>
-      <c r="F6" s="11">
-        <v>0.92</v>
+      <c r="F6" s="15">
+        <v>0.9689079666666668</v>
       </c>
       <c r="G6" s="5">
         <v>0.012248600656038687</v>
@@ -3833,10 +3904,13 @@
       <c r="I6" s="5">
         <v>0.006666666666666821</v>
       </c>
-      <c r="J6" s="5">
-        <f>10^-G6</f>
+      <c r="J6" s="14">
+        <f>10^-H6</f>
       </c>
       <c r="K6" s="3"/>
+      <c r="L6" s="15">
+        <v>0.9689079666666668</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="5">
@@ -3854,8 +3928,8 @@
       <c r="E7" s="5">
         <v>0.09620250054500204</v>
       </c>
-      <c r="F7" s="11">
-        <v>0.91</v>
+      <c r="F7" s="15">
+        <f>AVERAGE(F6,F8)</f>
       </c>
       <c r="G7" s="5">
         <v>0.14177843598383005</v>
@@ -3866,10 +3940,13 @@
       <c r="I7" s="5">
         <v>0.0033333333333332624</v>
       </c>
-      <c r="J7" s="5">
-        <f>10^-G7</f>
+      <c r="J7" s="14">
+        <f>10^-H7</f>
       </c>
       <c r="K7" s="3"/>
+      <c r="L7" s="15">
+        <v>1.0654959333333334</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="4">
@@ -3887,7 +3964,7 @@
       <c r="E8" s="5">
         <v>0.03272289378673253</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="13">
         <v>0.8997685</v>
       </c>
       <c r="G8" s="5">
@@ -3899,10 +3976,13 @@
       <c r="I8" s="5">
         <v>6.2803698347351e-16</v>
       </c>
-      <c r="J8" s="5">
-        <f>10^-G8</f>
+      <c r="J8" s="14">
+        <f>10^-H8</f>
       </c>
       <c r="K8" s="3"/>
+      <c r="L8" s="13">
+        <v>0.8997685</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="5">
@@ -3920,8 +4000,8 @@
       <c r="E9" s="5">
         <v>0.04058883261850885</v>
       </c>
-      <c r="F9" s="5">
-        <v>0.9</v>
+      <c r="F9" s="15">
+        <v>0.9534774666666667</v>
       </c>
       <c r="G9" s="5">
         <v>0.0007209760891396707</v>
@@ -3932,10 +4012,13 @@
       <c r="I9" s="5">
         <v>0.006666666666666821</v>
       </c>
-      <c r="J9" s="5">
-        <f>10^-G9</f>
+      <c r="J9" s="14">
+        <f>10^-H9</f>
       </c>
       <c r="K9" s="3"/>
+      <c r="L9" s="15">
+        <v>0.9534774666666667</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="4">
@@ -3953,8 +4036,8 @@
       <c r="E10" s="5">
         <v>0.026439427628701346</v>
       </c>
-      <c r="F10" s="5">
-        <v>0.9</v>
+      <c r="F10" s="15">
+        <v>0.9278216666666665</v>
       </c>
       <c r="G10" s="5">
         <v>0.0035484659602582165</v>
@@ -3965,23 +4048,49 @@
       <c r="I10" s="5">
         <v>0.00881917103688206</v>
       </c>
-      <c r="J10" s="5">
-        <f>10^-G10</f>
+      <c r="J10" s="14">
+        <f>10^-H10</f>
       </c>
       <c r="K10" s="3"/>
+      <c r="L10" s="15">
+        <v>0.9278216666666665</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
+      <c r="A11" s="5">
+        <v>99.5</v>
+      </c>
+      <c r="B11" s="5">
+        <v>1.192995</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.030650542817379306</v>
+      </c>
+      <c r="D11" s="5">
+        <v>3.2709333333333332</v>
+      </c>
+      <c r="E11" s="5">
+        <v>0.16515569758396006</v>
+      </c>
+      <c r="F11" s="13">
+        <v>0.9482218666666666</v>
+      </c>
+      <c r="G11" s="5">
+        <v>0.017242691340713382</v>
+      </c>
+      <c r="H11" s="5">
+        <v>6.383333333333333</v>
+      </c>
+      <c r="I11" s="5">
+        <v>0.0033333333333332624</v>
+      </c>
+      <c r="J11" s="14">
+        <f>10^-H11</f>
+      </c>
       <c r="K11" s="6"/>
+      <c r="L11" s="13">
+        <v>0.9482218666666666</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>